<commit_message>
Deployed b0ae9a0 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/API_workshop_template.xlsx
+++ b/API_workshop_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amsuni-my.sharepoint.com/personal/j_c_specker_uva_nl/Documents/Postdoc/PREMIER/ePiE/Workshop/mkdocs_manual/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{BCA84A6C-91EE-C24A-AC5C-448E9FF48EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E958C71-862C-4B81-93B8-969E63B7B90C}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{BCA84A6C-91EE-C24A-AC5C-448E9FF48EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A1662A5-3CF0-4A37-BEA5-D435DF973B36}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="result_template" sheetId="4" r:id="rId1"/>
@@ -113,9 +113,6 @@
     <t>NONE</t>
   </si>
   <si>
-    <t>MISSING</t>
-  </si>
-  <si>
     <t>Average Flow</t>
   </si>
   <si>
@@ -126,6 +123,9 @@
   </si>
   <si>
     <t>Rhine 1</t>
+  </si>
+  <si>
+    <t>6.21</t>
   </si>
 </sst>
 </file>
@@ -209,10 +209,10 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Good" xfId="2" builtinId="26"/>
@@ -497,30 +497,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FD6692C-546F-AA48-8DC7-482D45DE9EB1}">
   <dimension ref="A1:S27"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="26.21875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="12.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="20.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="21.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="11.44140625" style="1"/>
+    <col min="2" max="2" width="7.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.81640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="18.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.1796875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="20.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="21.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="11.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -579,7 +579,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -602,16 +602,16 @@
         <v>2019</v>
       </c>
       <c r="K2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L2">
         <v>107287</v>
       </c>
       <c r="M2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -634,16 +634,16 @@
         <v>2019</v>
       </c>
       <c r="K3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L3">
         <v>107287</v>
       </c>
       <c r="M3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -666,16 +666,16 @@
         <v>2019</v>
       </c>
       <c r="K4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L4">
         <v>107287</v>
       </c>
       <c r="M4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -698,16 +698,16 @@
         <v>2019</v>
       </c>
       <c r="K5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L5">
         <v>107287</v>
       </c>
       <c r="M5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -730,16 +730,16 @@
         <v>2019</v>
       </c>
       <c r="K6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L6">
         <v>107287</v>
       </c>
       <c r="M6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -762,16 +762,16 @@
         <v>2019</v>
       </c>
       <c r="K7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L7">
         <v>107287</v>
       </c>
       <c r="M7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -794,16 +794,16 @@
         <v>2019</v>
       </c>
       <c r="K8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L8">
         <v>124863</v>
       </c>
       <c r="M8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -826,16 +826,16 @@
         <v>2019</v>
       </c>
       <c r="K9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L9">
         <v>124863</v>
       </c>
       <c r="M9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -858,16 +858,16 @@
         <v>2019</v>
       </c>
       <c r="K10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L10">
         <v>124863</v>
       </c>
       <c r="M10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -890,16 +890,16 @@
         <v>2019</v>
       </c>
       <c r="K11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L11">
         <v>124863</v>
       </c>
       <c r="M11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -922,16 +922,16 @@
         <v>2019</v>
       </c>
       <c r="K12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L12">
         <v>124863</v>
       </c>
       <c r="M12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -954,16 +954,16 @@
         <v>2019</v>
       </c>
       <c r="K13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L13">
         <v>124863</v>
       </c>
       <c r="M13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -986,10 +986,10 @@
         <v>2019</v>
       </c>
       <c r="K14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1012,10 +1012,10 @@
         <v>2019</v>
       </c>
       <c r="K15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>22</v>
       </c>
       <c r="H16" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I16">
         <v>0.2</v>
@@ -1038,10 +1038,12 @@
         <v>2019</v>
       </c>
       <c r="K16" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+      <c r="L16"/>
+      <c r="M16"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1055,7 +1057,7 @@
         <v>22</v>
       </c>
       <c r="H17" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I17">
         <v>0.2</v>
@@ -1064,10 +1066,12 @@
         <v>2019</v>
       </c>
       <c r="K17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+      <c r="L17"/>
+      <c r="M17"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1090,10 +1094,10 @@
         <v>2019</v>
       </c>
       <c r="K18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1116,10 +1120,10 @@
         <v>2019</v>
       </c>
       <c r="K19" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1142,10 +1146,10 @@
         <v>2019</v>
       </c>
       <c r="K20" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1168,10 +1172,10 @@
         <v>2019</v>
       </c>
       <c r="K21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1197,10 +1201,10 @@
         <v>2019</v>
       </c>
       <c r="K22" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1226,10 +1230,10 @@
         <v>2019</v>
       </c>
       <c r="K23" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1255,10 +1259,10 @@
         <v>2019</v>
       </c>
       <c r="K24" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1284,10 +1288,10 @@
         <v>2019</v>
       </c>
       <c r="K25" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1313,10 +1317,10 @@
         <v>2019</v>
       </c>
       <c r="K26" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1342,7 +1346,7 @@
         <v>2019</v>
       </c>
       <c r="K27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 2b4f530 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/API_workshop_template.xlsx
+++ b/API_workshop_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amsuni-my.sharepoint.com/personal/j_c_specker_uva_nl/Documents/Postdoc/PREMIER/ePiE/Workshop/mkdocs_manual/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{BCA84A6C-91EE-C24A-AC5C-448E9FF48EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A1662A5-3CF0-4A37-BEA5-D435DF973B36}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{BCA84A6C-91EE-C24A-AC5C-448E9FF48EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27DFBE04-8E79-4D41-A292-F3BA8F27329B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="29">
   <si>
     <t>API</t>
   </si>
@@ -123,9 +123,6 @@
   </si>
   <si>
     <t>Rhine 1</t>
-  </si>
-  <si>
-    <t>6.21</t>
   </si>
 </sst>
 </file>
@@ -231,6 +228,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1028,8 +1029,8 @@
       <c r="D16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H16" t="s">
-        <v>29</v>
+      <c r="H16">
+        <v>6.21</v>
       </c>
       <c r="I16">
         <v>0.2</v>
@@ -1056,8 +1057,8 @@
       <c r="D17" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H17" t="s">
-        <v>29</v>
+      <c r="H17">
+        <v>6.21</v>
       </c>
       <c r="I17">
         <v>0.2</v>

</xml_diff>